<commit_message>
Rebuild group 2 (Loom B + CAN) from the wire lists: B-cabin, B-engine, CAN, WheelSpeed-Rear
Wheel-speed random ids renamed to plain names (both files).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/WheelSpeed-Front-pinouts.xlsx
+++ b/docs/harness/wirelist/WheelSpeed-Front-pinouts.xlsx
@@ -872,7 +872,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
@@ -952,7 +952,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>e7gavP</t>
+          <t>w_ws_f_shield</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>splice SvhsQx (Sensor screen join)</t>
+          <t>splice sp_ws_f_shield (Sensor screen join)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild group 2 (Loom B + CAN) from the wire lists: B-cabin, B-engine, CAN, WheelSpeed-Rear (#343)
Wheel-speed random ids renamed to plain names (both files).

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/WheelSpeed-Front-pinouts.xlsx
+++ b/docs/harness/wirelist/WheelSpeed-Front-pinouts.xlsx
@@ -872,7 +872,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
@@ -952,7 +952,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>e7gavP</t>
+          <t>w_ws_f_shield</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>splice SvhsQx (Sensor screen join)</t>
+          <t>splice sp_ws_f_shield (Sensor screen join)</t>
         </is>
       </c>
     </row>

</xml_diff>